<commit_message>
feat: initialize Prisma schema, implement finance bot service, and add CMR Excel template
</commit_message>
<xml_diff>
--- a/backend/templates/cmr_template.xlsx
+++ b/backend/templates/cmr_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{135E1AF9-EDB7-4F4F-B8D7-5E68D5DB56A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7704602-DE8E-4831-B0CC-148AC1C9099A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -785,7 +785,7 @@
       <c r="BD1" s="4"/>
       <c r="BE1" s="4"/>
     </row>
-    <row r="2" spans="2:57" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:57" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3"/>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -2305,7 +2305,7 @@
       <c r="BD27" s="2"/>
       <c r="BE27" s="2"/>
     </row>
-    <row r="28" spans="2:57" ht="3" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:57" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="28"/>
       <c r="C28" s="18"/>
       <c r="D28" s="18"/>
@@ -3597,7 +3597,7 @@
       <c r="BD47" s="26"/>
       <c r="BE47" s="26"/>
     </row>
-    <row r="48" spans="2:57" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:57" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="26"/>
       <c r="C48" s="26"/>
       <c r="D48" s="26"/>
@@ -4643,7 +4643,7 @@
       <c r="BD65" s="26"/>
       <c r="BE65" s="26"/>
     </row>
-    <row r="66" spans="2:57" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:57" ht="8.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="28"/>
       <c r="C66" s="28"/>
       <c r="D66" s="26"/>

</xml_diff>